<commit_message>
feat: add TrackingPage component for order tracking functionality
- Implemented TrackingPage to display order status and details.
- Added polling mechanism to refresh order status until it reaches a terminal state.
- Integrated error handling for order loading and display appropriate messages.

feat: create customer session management for storing customer name

- Added functions to read, write, and clear customer name in session storage.
- Implemented session expiration logic to manage customer name validity.

chore: add menu.xlsx file to the prisma directory
</commit_message>
<xml_diff>
--- a/server/prisma/menu.xlsx
+++ b/server/prisma/menu.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e5f99169480edbd6/Documents/Projects/pos-mavera/server/prisma/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Documents\pos-mavera\server\prisma\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{C133832B-8567-4B2D-B1FE-E55022C08DC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB396AA4-FD63-411A-AE57-F80F1FFD1D69}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{759DA2EE-1EC4-4061-A007-DDE17940356A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="600" yWindow="-120" windowWidth="28320" windowHeight="16440" xr2:uid="{B41294D9-DB93-42D4-9FB6-27DBB18C0353}"/>
+    <workbookView xWindow="3795" yWindow="3075" windowWidth="21060" windowHeight="11715" xr2:uid="{4047A78F-7173-4BD3-AF5D-8899BDFC65FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Menu" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <author>OpenAI</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{62205418-3400-4ABB-8A54-F93E9D201195}">
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{A423DA09-383B-4FFD-A27D-65A3EC2516F1}">
       <text>
         <r>
           <rPr>
@@ -58,7 +58,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{2EE9C218-DD42-4D0F-A9FB-9482742249CE}">
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{444F21E0-6328-484E-BBE0-C1268959571E}">
       <text>
         <r>
           <rPr>
@@ -72,7 +72,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{E1B14851-BEC1-49CA-88D4-D09D58EC62FE}">
+    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{CFC36F47-CF82-4F15-976E-E8E92BD76A24}">
       <text>
         <r>
           <rPr>
@@ -86,7 +86,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{2D709147-CC5B-4AA3-95D4-C4ECD55F8125}">
+    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{5B784240-7ED6-4440-AC18-77C7F40BBB4D}">
       <text>
         <r>
           <rPr>
@@ -100,7 +100,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{E4F77AC6-9275-47B4-937F-F2F562D2B6DC}">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{C1AE0CD3-7CB0-4255-907C-890996AA08CE}">
       <text>
         <r>
           <rPr>
@@ -114,7 +114,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{5E256D50-6C2B-49B5-B4A8-6B27A807B915}">
+    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{1B6CDE46-D533-4690-B8A1-D188CE287DDC}">
       <text>
         <r>
           <rPr>
@@ -128,7 +128,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{90854658-5061-4346-9F4D-254EB3237BE9}">
+    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{4F06244B-2194-4D8F-B84F-A035F08F8744}">
       <text>
         <r>
           <rPr>
@@ -142,7 +142,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{F0E8E97B-DC2A-474E-8079-3BA6F15C4F39}">
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{48F81CF5-50F3-47F4-B05D-B5675FC58C12}">
       <text>
         <r>
           <rPr>
@@ -161,7 +161,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="66">
   <si>
     <t>name</t>
   </si>
@@ -202,12 +202,21 @@
     <t>Paket A Keju</t>
   </si>
   <si>
+    <t>https://i.gojekapi.com/darkroom/gofood-indonesia/v2/images/uploads/09f97aba-47b0-4e89-8eb8-a4c92b46e094_Go-Biz_20230302_170707.jpeg?auto=format</t>
+  </si>
+  <si>
     <t>Paket A Mentai</t>
   </si>
   <si>
+    <t>https://kewpie.co.id/storage/recipes/featured-images/ab7b10a9-8010-4641-b0e1-4ab002ac6821.webp</t>
+  </si>
+  <si>
     <t>Paket A Mozzarela</t>
   </si>
   <si>
+    <t>https://asset.kompas.com/crops/TD_6D9lW6q-RcRpFJxTbyRvFZC0=/0x0:1000x667/1200x800/data/photo/2021/02/23/6034a60abb22b.jpg</t>
+  </si>
+  <si>
     <t>Paket B</t>
   </si>
   <si>
@@ -247,58 +256,106 @@
     <t>Tahu/Tempe</t>
   </si>
   <si>
+    <t>https://d1bpj0tv6vfxyp.cloudfront.net/articles/3be14058-960e-4007-abc1-03e949ccd01b_article_image_url.webp</t>
+  </si>
+  <si>
     <t>Tahu/Tempe Geprek</t>
   </si>
   <si>
     <t>Terong Penyet</t>
   </si>
   <si>
+    <t>https://www.finnafood.com/blog/wp-content/uploads/2022/04/terong-penyet.jpg</t>
+  </si>
+  <si>
     <t>Telur Dadar/Ceplok</t>
   </si>
   <si>
+    <t>https://www.dapurkobe.co.id/wp-content/uploads/nasi-telur-sentosa.jpg</t>
+  </si>
+  <si>
     <t>Sate Kulit</t>
   </si>
   <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcTW4utHAjMXhf7aCYo-54J0JcbxOwKHcPbJaYopnmBefg&amp;s=10</t>
+  </si>
+  <si>
     <t>Nasi Putih</t>
   </si>
   <si>
+    <t>https://drivethru.klikindomaret.com/ttlv/wp-content/uploads/sites/29/2020/09/Nasi-1.jpg</t>
+  </si>
+  <si>
     <t>Nasi Jeruk</t>
   </si>
   <si>
+    <t>https://asset.kompas.com/crops/KSmDxz9X-Qobx23Bp614jx73HqA=/3x0:700x465/1200x800/data/photo/2020/09/08/5f577fce97a7f.jpg</t>
+  </si>
+  <si>
     <t>Nasi Nori</t>
   </si>
   <si>
+    <t>https://img-global.cpcdn.com/recipes/981845095cb2c39f/1200x630cq80/photo.jpg</t>
+  </si>
+  <si>
     <t>Sambal</t>
   </si>
   <si>
+    <t>https://asset.kompas.com/crops/T5tcZX2QbELoIvtZeyVXOIq_KZI=/0x0:1000x667/1200x800/data/photo/2023/07/06/64a628ed595eb.jpeg</t>
+  </si>
+  <si>
     <t>Air Putih</t>
   </si>
   <si>
     <t>Minuman</t>
   </si>
   <si>
+    <t>https://image.astronauts.cloud/product-images/2026/7/OctZ1a051d37a1f01_cae11c6d-318f-4ada-bd08-17fff072d013_900x900.jpg</t>
+  </si>
+  <si>
     <t>Air Es</t>
   </si>
   <si>
+    <t>nnti delete</t>
+  </si>
+  <si>
     <t>Teh Tawar</t>
   </si>
   <si>
+    <t>https://dcostseafood.id/wp-content/uploads/2021/12/Teh-tawar-manis.jpg</t>
+  </si>
+  <si>
     <t>Es Teh Tawar</t>
   </si>
   <si>
+    <t>https://png.pngtree.com/png-clipart/20250823/original/pngtree-cold-sweet-tea-in-plastic-cup-png-image_21740884.png</t>
+  </si>
+  <si>
     <t>Es Teh Manis</t>
   </si>
   <si>
     <t>Es Jeruk Manis</t>
   </si>
   <si>
+    <t>https://png.pngtree.com/png-clipart/20250108/original/pngtree-icy-orange-drink-with-whole-and-half-png-image_19413745.png</t>
+  </si>
+  <si>
     <t>Es Lemon Tea</t>
   </si>
   <si>
+    <t>https://png.pngtree.com/png-clipart/20241208/original/pngtree-summer-iced-lemon-tea-png-image_17735822.png</t>
+  </si>
+  <si>
     <t>Es Jeruk Nipis</t>
   </si>
   <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcS1jtlQ8xlXC2cH4BSb8yVtzwzVU2uURHk8uZck3KdH2lWRC8ODgYc2ofPb&amp;s=10</t>
+  </si>
+  <si>
     <t>Es Teh Tarik</t>
+  </si>
+  <si>
+    <t>https://asset.kompas.com/crops/hsrnlGnJjSvQmAEyoV_dmwBbUi4=/120x80:1000x667/1200x800/data/photo/2023/10/18/652fcf5eb1b28.jpg</t>
   </si>
   <si>
     <t>Air Mineral</t>
@@ -321,7 +378,6 @@
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -676,7 +732,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4940337-AEE2-4818-8A6D-4C701CE1CE8C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{961CE7DF-BD01-430B-BD5A-CFC7AF8A53ED}">
   <dimension ref="A1:H36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -742,7 +798,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -756,7 +812,7 @@
         <v>10</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F3" s="2" t="b">
         <v>1</v>
@@ -768,9 +824,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>9</v>
@@ -782,7 +838,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F4" s="2" t="b">
         <v>1</v>
@@ -794,9 +850,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>9</v>
@@ -808,7 +864,7 @@
         <v>10</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F5" s="2" t="b">
         <v>1</v>
@@ -822,7 +878,7 @@
     </row>
     <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>9</v>
@@ -846,9 +902,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>9</v>
@@ -860,7 +916,7 @@
         <v>10</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F7" s="2" t="b">
         <v>1</v>
@@ -872,9 +928,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>9</v>
@@ -886,7 +942,7 @@
         <v>10</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F8" s="2" t="b">
         <v>1</v>
@@ -898,9 +954,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>9</v>
@@ -912,7 +968,7 @@
         <v>10</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F9" s="2" t="b">
         <v>1</v>
@@ -926,7 +982,7 @@
     </row>
     <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>9</v>
@@ -950,9 +1006,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>9</v>
@@ -964,7 +1020,7 @@
         <v>10</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F11" s="2" t="b">
         <v>1</v>
@@ -976,9 +1032,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>9</v>
@@ -990,7 +1046,7 @@
         <v>10</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F12" s="2" t="b">
         <v>1</v>
@@ -1002,9 +1058,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>9</v>
@@ -1016,7 +1072,7 @@
         <v>10</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F13" s="2" t="b">
         <v>1</v>
@@ -1054,12 +1110,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C15" s="4">
         <v>19000</v>
@@ -1068,7 +1124,7 @@
         <v>10</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F15" s="2" t="b">
         <v>1</v>
@@ -1080,12 +1136,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C16" s="4">
         <v>20000</v>
@@ -1094,7 +1150,7 @@
         <v>10</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F16" s="2" t="b">
         <v>1</v>
@@ -1106,12 +1162,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C17" s="4">
         <v>22000</v>
@@ -1120,7 +1176,7 @@
         <v>10</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F17" s="2" t="b">
         <v>1</v>
@@ -1132,12 +1188,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="C18" s="4">
         <v>1000</v>
@@ -1146,7 +1202,7 @@
         <v>10</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="F18" s="2" t="b">
         <v>1</v>
@@ -1158,12 +1214,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C19" s="4">
         <v>3000</v>
@@ -1172,7 +1228,7 @@
         <v>10</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="F19" s="2" t="b">
         <v>1</v>
@@ -1186,10 +1242,10 @@
     </row>
     <row r="20" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C20" s="4">
         <v>6000</v>
@@ -1198,7 +1254,7 @@
         <v>10</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F20" s="2" t="b">
         <v>1</v>
@@ -1212,10 +1268,10 @@
     </row>
     <row r="21" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C21" s="4">
         <v>5000</v>
@@ -1224,7 +1280,7 @@
         <v>10</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="F21" s="2" t="b">
         <v>1</v>
@@ -1236,12 +1292,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C22" s="4">
         <v>4000</v>
@@ -1250,7 +1306,7 @@
         <v>10</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="F22" s="2" t="b">
         <v>1</v>
@@ -1264,10 +1320,10 @@
     </row>
     <row r="23" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C23" s="4">
         <v>5000</v>
@@ -1276,7 +1332,7 @@
         <v>10</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="F23" s="2" t="b">
         <v>1</v>
@@ -1288,12 +1344,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C24" s="4">
         <v>6000</v>
@@ -1302,7 +1358,7 @@
         <v>10</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="F24" s="2" t="b">
         <v>1</v>
@@ -1314,12 +1370,12 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C25" s="4">
         <v>8000</v>
@@ -1328,7 +1384,7 @@
         <v>10</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="F25" s="2" t="b">
         <v>1</v>
@@ -1340,12 +1396,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C26" s="4">
         <v>3000</v>
@@ -1354,7 +1410,7 @@
         <v>10</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="F26" s="2" t="b">
         <v>1</v>
@@ -1366,12 +1422,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C27" s="4">
         <v>1000</v>
@@ -1380,7 +1436,7 @@
         <v>10</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="F27" s="2" t="b">
         <v>1</v>
@@ -1392,12 +1448,12 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C28" s="4">
         <v>2000</v>
@@ -1406,7 +1462,7 @@
         <v>10</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>11</v>
+        <v>51</v>
       </c>
       <c r="F28" s="2" t="b">
         <v>1</v>
@@ -1418,12 +1474,12 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C29" s="4">
         <v>2000</v>
@@ -1432,7 +1488,7 @@
         <v>10</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>11</v>
+        <v>53</v>
       </c>
       <c r="F29" s="2" t="b">
         <v>1</v>
@@ -1444,12 +1500,12 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C30" s="4">
         <v>3000</v>
@@ -1458,7 +1514,7 @@
         <v>10</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>11</v>
+        <v>55</v>
       </c>
       <c r="F30" s="2" t="b">
         <v>1</v>
@@ -1470,12 +1526,12 @@
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C31" s="4">
         <v>5000</v>
@@ -1484,7 +1540,7 @@
         <v>10</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>11</v>
+        <v>55</v>
       </c>
       <c r="F31" s="2" t="b">
         <v>1</v>
@@ -1496,12 +1552,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C32" s="4">
         <v>8000</v>
@@ -1510,7 +1566,7 @@
         <v>10</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>11</v>
+        <v>58</v>
       </c>
       <c r="F32" s="2" t="b">
         <v>1</v>
@@ -1522,12 +1578,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C33" s="4">
         <v>8000</v>
@@ -1536,7 +1592,7 @@
         <v>10</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>11</v>
+        <v>60</v>
       </c>
       <c r="F33" s="2" t="b">
         <v>1</v>
@@ -1548,12 +1604,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C34" s="4">
         <v>8000</v>
@@ -1562,7 +1618,7 @@
         <v>10</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>11</v>
+        <v>62</v>
       </c>
       <c r="F34" s="2" t="b">
         <v>1</v>
@@ -1574,12 +1630,12 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C35" s="4">
         <v>8000</v>
@@ -1588,7 +1644,7 @@
         <v>10</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>11</v>
+        <v>64</v>
       </c>
       <c r="F35" s="2" t="b">
         <v>1</v>
@@ -1600,12 +1656,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C36" s="4">
         <v>5000</v>
@@ -1614,7 +1670,7 @@
         <v>10</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="F36" s="2" t="b">
         <v>1</v>
@@ -1629,13 +1685,13 @@
   </sheetData>
   <autoFilter ref="A1:H501" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <dataValidations count="3">
-    <dataValidation type="list" errorTitle="Nilai tidak valid" error="Pilih TRUE atau FALSE." promptTitle="Boolean" prompt="Pilih TRUE atau FALSE." sqref="F2:G17 F37:G501 F18:F36 G19:G36" xr:uid="{932E6B9E-A482-41B5-A6A4-687FE3989669}">
+    <dataValidation type="list" errorTitle="Nilai tidak valid" error="Pilih TRUE atau FALSE." promptTitle="Boolean" prompt="Pilih TRUE atau FALSE." sqref="F2:G17 F37:G501 F18:F36 G19:G36" xr:uid="{9F0A27EC-F63C-455A-8439-BB9CFDADF9FA}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" sqref="H2:H501" xr:uid="{603ACC0C-3078-4ABC-BCA4-B2D88E862632}">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" sqref="H2:H501" xr:uid="{BECC3595-B234-4409-8994-2C2ABBA1C50A}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThan" errorTitle="Harga tidak valid" error="Harga harus berupa bilangan bulat lebih dari 0." sqref="C2:C501" xr:uid="{30A37A38-C5CD-40FA-81F3-5E2207803709}">
+    <dataValidation type="whole" operator="greaterThan" errorTitle="Harga tidak valid" error="Harga harus berupa bilangan bulat lebih dari 0." sqref="C2:C501" xr:uid="{B1BD1181-304B-4957-956B-FB2D5A32A3F4}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: implement payment attempt eligibility checks and add tests for payment functionality
</commit_message>
<xml_diff>
--- a/server/prisma/menu.xlsx
+++ b/server/prisma/menu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Documents\pos-mavera\server\prisma\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{759DA2EE-1EC4-4061-A007-DDE17940356A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E22859E7-6BE2-4FAC-9777-7D10E733826D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3795" yWindow="3075" windowWidth="21060" windowHeight="11715" xr2:uid="{4047A78F-7173-4BD3-AF5D-8899BDFC65FD}"/>
+    <workbookView xWindow="19810" yWindow="610" windowWidth="18700" windowHeight="12220" xr2:uid="{4047A78F-7173-4BD3-AF5D-8899BDFC65FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Menu" sheetId="1" r:id="rId1"/>
@@ -365,7 +365,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -378,6 +378,14 @@
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -411,10 +419,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -431,8 +440,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1201,7 +1214,7 @@
       <c r="D18" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F18" s="2" t="b">
@@ -1279,7 +1292,7 @@
       <c r="D21" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="6" t="s">
         <v>36</v>
       </c>
       <c r="F21" s="2" t="b">
@@ -1305,7 +1318,7 @@
       <c r="D22" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E22" s="6" t="s">
         <v>38</v>
       </c>
       <c r="F22" s="2" t="b">
@@ -1331,7 +1344,7 @@
       <c r="D23" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="E23" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F23" s="2" t="b">
@@ -1487,7 +1500,7 @@
       <c r="D29" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="E29" s="6" t="s">
         <v>53</v>
       </c>
       <c r="F29" s="2" t="b">
@@ -1513,7 +1526,7 @@
       <c r="D30" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="E30" s="6" t="s">
         <v>55</v>
       </c>
       <c r="F30" s="2" t="b">
@@ -1565,7 +1578,7 @@
       <c r="D32" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="E32" s="6" t="s">
         <v>58</v>
       </c>
       <c r="F32" s="2" t="b">
@@ -1643,7 +1656,7 @@
       <c r="D35" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="E35" s="6" t="s">
         <v>64</v>
       </c>
       <c r="F35" s="2" t="b">
@@ -1695,7 +1708,17 @@
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="E18" r:id="rId1" xr:uid="{342125F6-D92A-43D5-8DCF-36CF87C011B5}"/>
+    <hyperlink ref="E21" r:id="rId2" xr:uid="{387E0FDD-048E-4A9D-8BF0-CCBA1B985DF6}"/>
+    <hyperlink ref="E22" r:id="rId3" xr:uid="{27929ED9-3F94-40E1-B3D5-CADEBE935BB6}"/>
+    <hyperlink ref="E23" r:id="rId4" xr:uid="{3F62F01D-34FC-4D68-93B3-FBA628B56799}"/>
+    <hyperlink ref="E29" r:id="rId5" xr:uid="{C232747E-B5B1-42B5-AC5D-C898269B9643}"/>
+    <hyperlink ref="E30" r:id="rId6" xr:uid="{6701DB77-0B6C-46DE-90AA-A7FCF5450B74}"/>
+    <hyperlink ref="E32" r:id="rId7" xr:uid="{AE5F0FEF-4F06-4BCF-9DD0-C758823CFFAE}"/>
+    <hyperlink ref="E35" r:id="rId8" xr:uid="{45D95F43-7DA4-48AA-A711-29232D49EB2F}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing r:id="rId1"/>
+  <legacyDrawing r:id="rId9"/>
 </worksheet>
 </file>
</xml_diff>